<commit_message>
Custom sleeves and portfolios, the fee card, and the deck built in the house template (D164-D177)
- Custom sleeves and custom portfolios, with one PWA switch and fixed profile limits (D170-D173)
- The deck is built from a template's layout, placed by marks, with the strategic and fee slides restyled (D174-D176)
- Other Charges on the pricing row: FX sizes fixed at $5M and $1M, custody $5,000 unless set ($0 for GSBZ Custody); Download opens the card while any is missing, and a priced export refuses them missing (D177)
- No Proposal UID on a template deck: it goes in the workbook only
- The register gains the charges (schema 9)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RrbEDqpbzGybDjq7WZNesz
</commit_message>
<xml_diff>
--- a/dataTemplates/ProposalTool_DataTemplates.xlsx
+++ b/dataTemplates/ProposalTool_DataTemplates.xlsx
@@ -290,7 +290,7 @@
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <t>ShareClass (optional, text)
-Dis (distributing) or Acc (accumulating), and nothing else - a typo is refused on load. Leave blank, or drop the column, for a product that has no share class.</t>
+Distributing or Accumulating, and nothing else - a typo is refused on load. Leave blank, or drop the column, for a product that has no share class.</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
@@ -895,7 +895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -927,89 +927,64 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>The products and feeRates sheets fill the product catalogue and the fee card the first time the tool opens after it is installed or upgraded. After that the tool keeps both: a new file goes in through Import a file on the Repository's Catalogue or Fees tab, where what it would change is shown before anything does.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Save as</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Environment variable</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Format</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>What it feeds</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>saaPortfolios</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>saaPortfolios.csv</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>SCENARIO_SAA_SOURCE</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>CSV or XLSX</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Every strategic portfolio the tool can offer, one row per holding. The portfolio NAME is the key: it is parsed, never guessed.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>products</t>
+          <t>saaPortfolios</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>products.csv</t>
+          <t>saaPortfolios.csv</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>SCENARIO_PRODUCTS_SOURCE</t>
+          <t>SCENARIO_SAA_SOURCE</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>CSV</t>
+          <t>CSV or XLSX</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -1019,24 +994,24 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>The delivered product catalogue every sleeve picks from. Re-read whenever the file changes on disk.</t>
+          <t>Every strategic portfolio the tool can offer, one row per holding. The portfolio NAME is the key: it is parsed, never guessed.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>sleeves</t>
+          <t>products</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>sleeves.csv</t>
+          <t>products.csv</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>SCENARIO_SLEEVES_SEED</t>
+          <t>SCENARIO_PRODUCTS_SOURCE</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -1051,24 +1026,24 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>The starting sleeve library, one row per product in a sleeve. READ ONCE, on the first start against an empty sleeve database; after that the admin console is the source of truth and this file is not read again.</t>
+          <t>The delivered product catalogue every sleeve picks from. Re-read whenever the file changes on disk.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>sleeveRules</t>
+          <t>sleeves</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>sleeveRules.csv</t>
+          <t>sleeves.csv</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>SCENARIO_SLEEVES_RULES</t>
+          <t>SCENARIO_SLEEVES_SEED</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1083,24 +1058,24 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Which strategic portfolios each labelled edition on the sleeves sheet is for: one row per rule. An edition with several rows applies where ANY of them matches. A rule matches a portfolio when every filled cell contains the portfolio's value; a blank cell means any. Read with the sleeves sheet, once, on the first start; optional - a library with no editions needs no rules. Two editions of one name may not both claim a portfolio: the load refuses and names the clash.</t>
+          <t>The starting sleeve library, one row per product in a sleeve. READ ONCE, on the first start against an empty sleeve database; after that the admin console is the source of truth and this file is not read again.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>feeRates</t>
+          <t>sleeveRules</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>feeRates.csv</t>
+          <t>sleeveRules.csv</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>SCENARIO_FEES_SOURCE</t>
+          <t>SCENARIO_SLEEVES_RULES</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1115,138 +1090,171 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>The rate card: one row per cell. Deliver it through "feeTools --diff &lt;csv&gt;" then "--accept", which records the version and clears the placeholder flag the rail, the workbook and the bake manifest all read.</t>
+          <t>Which strategic portfolios each labelled edition on the sleeves sheet is for: one row per rule. An edition with several rows applies where ANY of them matches. A rule matches a portfolio when every filled cell contains the portfolio's value; a blank cell means any. Read with the sleeves sheet, once, on the first start; optional - a library with no editions needs no rules. Two editions of one name may not both claim a portfolio: the load refuses and names the clash.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>advisors</t>
+          <t>feeRates</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>advisors.xlsx (inside the package, beside advisors.py)</t>
+          <t>feeRates.csv</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>none - there is no override</t>
+          <t>SCENARIO_FEES_SOURCE</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>XLSX, first sheet</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>replace the packaged file</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>The Primary PWA directory behind the typeahead. A mandate's Primary PWA must equal a display string exactly, or creating a scenario is refused.</t>
+          <t>The rate card: one row per cell. Deliver it through "feeTools --diff &lt;csv&gt;" then "--accept", which records the version and clears the placeholder flag the rail, the workbook and the bake manifest all read.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>assetEstimates</t>
+          <t>advisors</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>assetEstimates.json</t>
+          <t>advisors.xlsx (inside the package, beside advisors.py)</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>SCENARIO_ASSET_ESTIMATES</t>
+          <t>none - there is no override</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>JSON (see note)</t>
+          <t>XLSX, first sheet</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>replace the packaged file</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>The per-asset long-term estimates behind the workbook's assumptions sheet, one block per currency-and-hedging slice. THE SERVICE READS JSON: fill this table in, then convert it - the shape is on the portfolioAnalytics sheet.</t>
+          <t>The Primary PWA directory behind the typeahead. A mandate's Primary PWA must equal a display string exactly, or creating a scenario is refused.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
+          <t>assetEstimates</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>assetEstimates.json</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>SCENARIO_ASSET_ESTIMATES</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>JSON (see note)</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>The per-asset long-term estimates behind the workbook's assumptions sheet, one block per currency-and-hedging slice. THE SERVICE READS JSON: fill this table in, then convert it - the shape is on the portfolioAnalytics sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
           <t>portfolioAnalytics</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>&lt;slice&gt;.json + manifest.json</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>SCENARIO_BAKED_DIR</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>JSON</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>The risk and return figures themselves. Generated, not typed - see that sheet.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Check your files with:</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>python -m cyrus_pmg.pmgService.scenario.bake --census        # the SAA extract: 0 unparsed, no unknown tickers</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>python -m cyrus_pmg.pmgService.scenario.sleeveTools --census # the sleeve library: no broken sleeves, no orphans</t>
+          <t>python -m cyrus_pmg.pmgService.scenario.bake --census        # the SAA extract: 0 unparsed, no unknown tickers</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
+          <t>python -m cyrus_pmg.pmgService.scenario.sleeveTools --census # the sleeve library: no broken sleeves, no orphans</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
           <t>python -m cyrus_pmg.pmgService.scenario.feeTools --census    # the rate card, and whether it is still a placeholder</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1918,7 +1926,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Dis (distributing) or Acc (accumulating), and nothing else - a typo is refused on load. Leave blank, or drop the column, for a product that has no share class.</t>
+          <t>Distributing or Accumulating, and nothing else - a typo is refused on load. Leave blank, or drop the column, for a product that has no share class.</t>
         </is>
       </c>
     </row>
@@ -3106,7 +3114,7 @@
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
@@ -3259,7 +3267,7 @@
       </c>
       <c r="I2" s="8" t="inlineStr">
         <is>
-          <t>Dis</t>
+          <t>Distributing</t>
         </is>
       </c>
       <c r="J2" s="8" t="inlineStr">
@@ -3356,7 +3364,7 @@
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
-          <t>Acc</t>
+          <t>Accumulating</t>
         </is>
       </c>
       <c r="J3" s="8" t="inlineStr">
@@ -4294,7 +4302,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Dis</t>
+          <t>Distributing</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -4356,7 +4364,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Dis</t>
+          <t>Distributing</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">

</xml_diff>

<commit_message>
The product Category, which bands the catalogue (D178) - Products gain an optional Category (headed Category, Catagory or Group), one of the categories the sleeves are built for; the catalogue bands by it, then by the sleeves that hold the product, else No category - The sleeve database gains the column (schema 9) - The catalogue's missing-products warning folds to one line with Show the list - The house template check takes a template without a cover marker to have its own cover - The re-seeding guide: adding the categories
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RrbEDqpbzGybDjq7WZNesz
</commit_message>
<xml_diff>
--- a/dataTemplates/ProposalTool_DataTemplates.xlsx
+++ b/dataTemplates/ProposalTool_DataTemplates.xlsx
@@ -277,59 +277,65 @@
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
+        <t>Category (optional, text)
+The sleeve category the catalogue groups the product under: one the library knows, spelled as it spells it, e.g. Public Equity - a typo is refused on import. The column may also be headed Catagory or Group. Blank for none.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
         <t>Style (yes, text)
 Free text. One of the five composition doughnuts groups by this.</t>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
+    <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <t>Vehicle (yes, text)
 Free text, e.g. SMA, Mutual Fund, ETF. A doughnut axis.</t>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <t>ShareClass (optional, text)
 Distributing or Accumulating, and nothing else - a typo is refused on load. Leave blank, or drop the column, for a product that has no share class.</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <t>Source (yes, text)
 Free text, e.g. Internal, External. A doughnut axis.</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <t>Liquidity (yes, text)
 Free text, e.g. Daily, Quarterly. A doughnut axis.</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
+    <comment ref="K1" authorId="0" shapeId="0">
       <text>
         <t>ExposureCurrency (yes, text)
 Free text, e.g. USD. A doughnut axis.</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
+    <comment ref="L1" authorId="0" shapeId="0">
       <text>
         <t>ProductCost (yes, number &gt;= 0)
 A PERCENT: 0.25 means 0.25%. Not a fraction.</t>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <t>FeeGroup (yes, text)
 One of the fee groups on the Valid values sheet. The set is defined by the feeRates sheet, so the two must agree.</t>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="N1" authorId="0" shapeId="0">
       <text>
         <t>DistributionYield (optional, number &gt;= 0)
 A PERCENT. Leave blank, or drop the column, if there is none.</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="O1" authorId="0" shapeId="0">
       <text>
         <t>MinimumInvestment (optional, number &gt;= 0)
 CURRENCY UNITS: 5000000 means $5m. Blank means no minimum. THIS BLOCKS THE EXPORT: a position below its product minimum refuses the download, so get these right.</t>
@@ -1616,7 +1622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1857,12 +1863,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Style</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>optional</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1872,7 +1878,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Free text. One of the five composition doughnuts groups by this.</t>
+          <t>The sleeve category the catalogue groups the product under: one the library knows, spelled as it spells it, e.g. Public Equity - a typo is refused on import. The column may also be headed Catagory or Group. Blank for none.</t>
         </is>
       </c>
     </row>
@@ -1884,7 +1890,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Vehicle</t>
+          <t>Style</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -1899,7 +1905,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Free text, e.g. SMA, Mutual Fund, ETF. A doughnut axis.</t>
+          <t>Free text. One of the five composition doughnuts groups by this.</t>
         </is>
       </c>
     </row>
@@ -1911,12 +1917,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>ShareClass</t>
+          <t>Vehicle</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>optional</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -1926,7 +1932,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Distributing or Accumulating, and nothing else - a typo is refused on load. Leave blank, or drop the column, for a product that has no share class.</t>
+          <t>Free text, e.g. SMA, Mutual Fund, ETF. A doughnut axis.</t>
         </is>
       </c>
     </row>
@@ -1938,12 +1944,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>ShareClass</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>optional</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1953,7 +1959,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Free text, e.g. Internal, External. A doughnut axis.</t>
+          <t>Distributing or Accumulating, and nothing else - a typo is refused on load. Leave blank, or drop the column, for a product that has no share class.</t>
         </is>
       </c>
     </row>
@@ -1965,7 +1971,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Liquidity</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -1980,7 +1986,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Free text, e.g. Daily, Quarterly. A doughnut axis.</t>
+          <t>Free text, e.g. Internal, External. A doughnut axis.</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1998,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>ExposureCurrency</t>
+          <t>Liquidity</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -2007,7 +2013,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Free text, e.g. USD. A doughnut axis.</t>
+          <t>Free text, e.g. Daily, Quarterly. A doughnut axis.</t>
         </is>
       </c>
     </row>
@@ -2019,7 +2025,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>ProductCost</t>
+          <t>ExposureCurrency</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -2029,12 +2035,12 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>number &gt;= 0</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>A PERCENT: 0.25 means 0.25%. Not a fraction.</t>
+          <t>Free text, e.g. USD. A doughnut axis.</t>
         </is>
       </c>
     </row>
@@ -2046,7 +2052,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>FeeGroup</t>
+          <t>ProductCost</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -2056,12 +2062,12 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>number &gt;= 0</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>One of the fee groups on the Valid values sheet. The set is defined by the feeRates sheet, so the two must agree.</t>
+          <t>A PERCENT: 0.25 means 0.25%. Not a fraction.</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2079,22 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>DistributionYield</t>
+          <t>FeeGroup</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>optional</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>number &gt;= 0</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>A PERCENT. Leave blank, or drop the column, if there is none.</t>
+          <t>One of the fee groups on the Valid values sheet. The set is defined by the feeRates sheet, so the two must agree.</t>
         </is>
       </c>
     </row>
@@ -2100,7 +2106,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>MinimumInvestment</t>
+          <t>DistributionYield</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -2115,34 +2121,34 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>CURRENCY UNITS: 5000000 means $5m. Blank means no minimum. THIS BLOCKS THE EXPORT: a position below its product minimum refuses the download, so get these right.</t>
+          <t>A PERCENT. Leave blank, or drop the column, if there is none.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>sleeves</t>
+          <t>products</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Variant</t>
+          <t>MinimumInvestment</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>optional</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>number &gt;= 0</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>One of the four implementation types on the Valid values sheet.</t>
+          <t>CURRENCY UNITS: 5000000 means $5m. Blank means no minimum. THIS BLOCKS THE EXPORT: a position below its product minimum refuses the download, so get these right.</t>
         </is>
       </c>
     </row>
@@ -2154,7 +2160,7 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Variant</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -2169,7 +2175,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>One of the seven sleeve categories on the Valid values sheet. Private Equity and Other Private Assets share the one combined category.</t>
+          <t>One of the four implementation types on the Valid values sheet.</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2187,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Sleeve</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -2191,12 +2197,12 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>text (&lt;= 80)</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>The sleeve name: what a PWA picks. Its editions share it. Unique within a variant and category together with the Edition.</t>
+          <t>One of the seven sleeve categories on the Valid values sheet. Private Equity and Other Private Assets share the one combined category.</t>
         </is>
       </c>
     </row>
@@ -2208,12 +2214,12 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Edition</t>
+          <t>Sleeve</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -2223,7 +2229,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>BLANK for the fallback edition, which applies wherever no other edition of the name does; or the desk's short label for an edition that is only for particular strategic portfolios ("GBP", "GBP ex-Alts"). A labelled edition must have rules on the sleeveRules sheet; a fallback must not. At most one fallback per name. The header without this column is still accepted: every row is then a fallback.</t>
+          <t>The sleeve name: what a PWA picks. Its editions share it. Unique within a variant and category together with the Edition.</t>
         </is>
       </c>
     </row>
@@ -2235,22 +2241,22 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>ProductId</t>
+          <t>Edition</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>text (&lt;= 80)</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Must exist in the products sheet.</t>
+          <t>BLANK for the fallback edition, which applies wherever no other edition of the name does; or the desk's short label for an edition that is only for particular strategic portfolios ("GBP", "GBP ex-Alts"). A labelled edition must have rules on the sleeveRules sheet; a fallback must not. At most one fallback per name. The header without this column is still accepted: every row is then a fallback.</t>
         </is>
       </c>
     </row>
@@ -2262,7 +2268,7 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Weight</t>
+          <t>ProductId</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -2272,24 +2278,24 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>A FRACTION. One edition's rows must sum to 1 within 0.000001.</t>
+          <t>Must exist in the products sheet.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>sleeveRules</t>
+          <t>sleeves</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Variant</t>
+          <t>Weight</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -2299,12 +2305,12 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>number</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>As on the sleeves sheet.</t>
+          <t>A FRACTION. One edition's rows must sum to 1 within 0.000001.</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2322,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Variant</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -2343,7 +2349,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Sleeve</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -2358,7 +2364,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>The sleeve name, exactly as on the sleeves sheet.</t>
+          <t>As on the sleeves sheet.</t>
         </is>
       </c>
     </row>
@@ -2370,7 +2376,7 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Edition</t>
+          <t>Sleeve</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
@@ -2385,7 +2391,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>The edition label, exactly as on the sleeves sheet. Never blank here: the fallback has no rules.</t>
+          <t>The sleeve name, exactly as on the sleeves sheet.</t>
         </is>
       </c>
     </row>
@@ -2397,12 +2403,12 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>Edition</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -2412,7 +2418,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>One or more currencies from the Valid values sheet, several separated by | ("GBP" or "GBP|EUR"). Blank means any currency.</t>
+          <t>The edition label, exactly as on the sleeves sheet. Never blank here: the fallback has no rules.</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2430,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>RiskLevel</t>
+          <t>Currency</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -2439,7 +2445,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>One or more risk levels from the Valid values sheet, several separated by | ("Moderate" or "Moderate|ModAgg"). Blank means any risk level.</t>
+          <t>One or more currencies from the Valid values sheet, several separated by | ("GBP" or "GBP|EUR"). Blank means any currency.</t>
         </is>
       </c>
     </row>
@@ -2451,7 +2457,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>AllocationType</t>
+          <t>RiskLevel</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -2466,24 +2472,24 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>One or more allocation types from the Valid values sheet, several separated by |, and NA for the all-equity book ("ex-Alts" or "Full|Core|ex-HFs|NA"). Blank means any. At least one of the three cells must be filled: a rule that constrains nothing is refused. Hedging and the real-assets exclusion are not rule fields.</t>
+          <t>One or more risk levels from the Valid values sheet, several separated by | ("Moderate" or "Moderate|ModAgg"). Blank means any risk level.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>feeRates</t>
+          <t>sleeveRules</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>schedule</t>
+          <t>AllocationType</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
@@ -2493,7 +2499,7 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>CASP (one rate for all) or RDR (a rate per fee group).</t>
+          <t>One or more allocation types from the Valid values sheet, several separated by |, and NA for the all-equity book ("ex-Alts" or "Full|Core|ex-HFs|NA"). Blank means any. At least one of the three cells must be filled: a rule that constrains nothing is refused. Hedging and the real-assets exclusion are not rule fields.</t>
         </is>
       </c>
     </row>
@@ -2505,12 +2511,12 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>feeGroup</t>
+          <t>schedule</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>yes for RDR</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
@@ -2520,7 +2526,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Blank for CASP. For RDR, the fee group. The distinct values here DEFINE the set the products sheet must use.</t>
+          <t>CASP (one rate for all) or RDR (a rate per fee group).</t>
         </is>
       </c>
     </row>
@@ -2532,12 +2538,12 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>tier</t>
+          <t>feeGroup</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>yes for RDR</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -2547,7 +2553,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Tier id, e.g. T1. Every row of a tier must carry the same edges.</t>
+          <t>Blank for CASP. For RDR, the fee group. The distinct values here DEFINE the set the products sheet must use.</t>
         </is>
       </c>
     </row>
@@ -2559,7 +2565,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>tierMin</t>
+          <t>tier</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -2569,12 +2575,12 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Top-account-size lower edge, CURRENCY UNITS. Inclusive.</t>
+          <t>Tier id, e.g. T1. Every row of a tier must carry the same edges.</t>
         </is>
       </c>
     </row>
@@ -2586,12 +2592,12 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>tierMax</t>
+          <t>tierMin</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
@@ -2601,7 +2607,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Upper edge, CURRENCY UNITS, exclusive. LEAVE IT EMPTY ON THE TOP TIER: an empty cell is how a tier says "and up", and the tier then reads as "$100m and up". Do not write Infinity, inf, or a very large number - all three are refused on load.</t>
+          <t>Top-account-size lower edge, CURRENCY UNITS. Inclusive.</t>
         </is>
       </c>
     </row>
@@ -2613,22 +2619,22 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>tierMax</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>number</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>Management or PMG.</t>
+          <t>Upper edge, CURRENCY UNITS, exclusive. LEAVE IT EMPTY ON THE TOP TIER: an empty cell is how a tier says "and up", and the tier then reads as "$100m and up". Do not write Infinity, inf, or a very large number - all three are refused on load.</t>
         </is>
       </c>
     </row>
@@ -2640,7 +2646,7 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>point</t>
+          <t>source</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
@@ -2655,7 +2661,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Floor, Target or Ceiling. A proposal prices at "&lt;source&gt; &lt;point&gt;", e.g. PMG Floor.</t>
+          <t>Management or PMG.</t>
         </is>
       </c>
     </row>
@@ -2667,7 +2673,7 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>rate</t>
+          <t>point</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -2677,24 +2683,24 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>number &gt;= 0</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>A PERCENT: 0.45 means 0.45%.</t>
+          <t>Floor, Target or Ceiling. A proposal prices at "&lt;source&gt; &lt;point&gt;", e.g. PMG Floor.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>advisors</t>
+          <t>feeRates</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>rate</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
@@ -2704,12 +2710,12 @@
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>number &gt;= 0</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>The advisor name as it should read.</t>
+          <t>A PERCENT: 0.45 means 0.45%.</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2727,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>office</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -2736,19 +2742,19 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>The office. The display string is "name - office" with an em dash.</t>
+          <t>The advisor name as it should read.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>assetEstimates</t>
+          <t>advisors</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Slice</t>
+          <t>office</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
@@ -2763,7 +2769,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>Currency and hedging, e.g. "USD|Hedged". Sixteen in all.</t>
+          <t>The office. The display string is "name - office" with an em dash.</t>
         </is>
       </c>
     </row>
@@ -2775,7 +2781,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>AnalyticsCurrency</t>
+          <t>Slice</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -2790,7 +2796,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>The currency the figures were actually computed in. Equal to the slice currency unless it was run in another, which the bake manifest then records.</t>
+          <t>Currency and hedging, e.g. "USD|Hedged". Sixteen in all.</t>
         </is>
       </c>
     </row>
@@ -2802,7 +2808,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>ReportingName</t>
+          <t>AnalyticsCurrency</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
@@ -2817,7 +2823,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>One of the 19 asset reporting names on the Valid values sheet.</t>
+          <t>The currency the figures were actually computed in. Equal to the slice currency unless it was run in another, which the bake manifest then records.</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2835,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>ReportingName</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -2844,7 +2850,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>That asset's category, as on the Valid values sheet.</t>
+          <t>One of the 19 asset reporting names on the Valid values sheet.</t>
         </is>
       </c>
     </row>
@@ -2856,7 +2862,7 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Lower</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
@@ -2866,12 +2872,12 @@
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>FRACTION: 0.006 means 0.6%. Lower bound of the risk-premium estimate.</t>
+          <t>That asset's category, as on the Valid values sheet.</t>
         </is>
       </c>
     </row>
@@ -2883,7 +2889,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Mean</t>
+          <t>Lower</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
@@ -2898,7 +2904,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>FRACTION. The central risk-premium estimate.</t>
+          <t>FRACTION: 0.006 means 0.6%. Lower bound of the risk-premium estimate.</t>
         </is>
       </c>
     </row>
@@ -2910,7 +2916,7 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Upper</t>
+          <t>Mean</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
@@ -2925,7 +2931,7 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>FRACTION. Upper bound.</t>
+          <t>FRACTION. The central risk-premium estimate.</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2943,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Volatility</t>
+          <t>Upper</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
@@ -2952,7 +2958,7 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>FRACTION.</t>
+          <t>FRACTION. Upper bound.</t>
         </is>
       </c>
     </row>
@@ -2964,7 +2970,7 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Sharpe</t>
+          <t>Volatility</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
@@ -2979,7 +2985,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>A ratio, not a percent.</t>
+          <t>FRACTION.</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2997,7 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>TotalReturn</t>
+          <t>Sharpe</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
@@ -3006,7 +3012,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>FRACTION.</t>
+          <t>A ratio, not a percent.</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3024,7 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>HedgingRatio</t>
+          <t>TotalReturn</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
@@ -3033,7 +3039,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>FRACTION: 1.0 means fully hedged.</t>
+          <t>FRACTION.</t>
         </is>
       </c>
     </row>
@@ -3045,7 +3051,7 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>From</t>
+          <t>HedgingRatio</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
@@ -3055,12 +3061,12 @@
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>number</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>ISO date, e.g. 1973-02-28. Start of the estimation window.</t>
+          <t>FRACTION: 1.0 means fully hedged.</t>
         </is>
       </c>
     </row>
@@ -3072,20 +3078,47 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>ISO date, e.g. 1973-02-28. Start of the estimation window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>assetEstimates</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
           <t>To</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="E56" s="5" t="inlineStr">
+      <c r="E57" s="5" t="inlineStr">
         <is>
           <t>ISO date. End of the estimation window.</t>
         </is>
@@ -4182,7 +4215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -4191,14 +4224,15 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="23" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
     <col width="23" customWidth="1" min="14" max="14"/>
+    <col width="23" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4224,50 +4258,55 @@
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
           <t>Style</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Vehicle</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>ShareClass</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Liquidity</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>ExposureCurrency</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>ProductCost</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>FeeGroup</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>DistributionYield</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>MinimumInvestment</t>
         </is>
@@ -4292,46 +4331,51 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
+          <t>Investment Grade Fixed Income</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>SMA</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Distributing</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Internal</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Daily</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="K2" s="3" t="n">
+      <c r="L2" s="3" t="n">
         <v>0.25</v>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>Core Active</t>
         </is>
       </c>
-      <c r="M2" s="3" t="n">
+      <c r="N2" s="3" t="n">
         <v>3.2</v>
       </c>
-      <c r="N2" s="3" t="n">
+      <c r="O2" s="3" t="n">
         <v>5000000</v>
       </c>
     </row>
@@ -4354,55 +4398,60 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
+          <t>Investment Grade Fixed Income</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>SMA</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Distributing</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Internal</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Daily</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="K3" s="3" t="n">
+      <c r="L3" s="3" t="n">
         <v>0.28</v>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Core Active</t>
         </is>
       </c>
-      <c r="M3" s="3" t="n">
+      <c r="N3" s="3" t="n">
         <v>4.8</v>
       </c>
-      <c r="N3" s="3" t="n">
+      <c r="O3" s="3" t="n">
         <v>5000000</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="L2:L5000" showErrorMessage="1" showDropDown="0" showInputMessage="1" allowBlank="1" errorTitle="Not a permitted value" error="Choose a value from the Valid values sheet." type="list">
+    <dataValidation sqref="M2:M5000" showErrorMessage="1" showDropDown="0" showInputMessage="1" allowBlank="1" errorTitle="Not a permitted value" error="Choose a value from the Valid values sheet." type="list">
       <formula1>'Valid values'!$H$2:$H$6</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G5000" showErrorMessage="1" showDropDown="0" showInputMessage="1" allowBlank="1" errorTitle="Not a permitted value" error="Choose a value from the Valid values sheet." type="list">
+    <dataValidation sqref="H2:H5000" showErrorMessage="1" showDropDown="0" showInputMessage="1" allowBlank="1" errorTitle="Not a permitted value" error="Choose a value from the Valid values sheet." type="list">
       <formula1>'Valid values'!$I$2:$I$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>